<commit_message>
fix: complete trial balance review controls
</commit_message>
<xml_diff>
--- a/frontend/public/template-files/trial-balance-review-workpaper-template.xlsx
+++ b/frontend/public/template-files/trial-balance-review-workpaper-template.xlsx
@@ -12,14 +12,14 @@
     <sheet sheetId="6" name="Lists" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Summary'!$A1:$H22</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Summary'!$A1:$H23</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="125">
   <si>
     <t>Trial Balance Review Workpaper</t>
   </si>
@@ -177,10 +177,10 @@
     <t>Prepaid Expenses</t>
   </si>
   <si>
-    <t>Other</t>
+    <t>Unresolved</t>
   </si>
   <si>
-    <t/>
+    <t>Classification support is unresolved</t>
   </si>
   <si>
     <t>1500</t>
@@ -190,6 +190,9 @@
   </si>
   <si>
     <t>Fixed Assets</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>1590</t>
@@ -336,6 +339,15 @@
     <t>Current Difference</t>
   </si>
   <si>
+    <t>Prior Debits</t>
+  </si>
+  <si>
+    <t>Prior Credits</t>
+  </si>
+  <si>
+    <t>Prior Difference</t>
+  </si>
+  <si>
     <t>Proposed Adjustments</t>
   </si>
   <si>
@@ -351,13 +363,16 @@
     <t>Unmapped Count</t>
   </si>
   <si>
+    <t>Unresolved Count</t>
+  </si>
+  <si>
     <t>Open Review Count</t>
   </si>
   <si>
     <t>Reviewer Notes</t>
   </si>
   <si>
-    <t>Resolve mapping, unusual-sign, and material-movement review items before sign-off. Proposed adjustments use positive debit and negative credit signs.</t>
+    <t>Resolve unresolved classification, mapping, unusual-sign, and material-movement items before sign-off. Proposed adjustments use positive debit and negative credit signs.</t>
   </si>
   <si>
     <t>Review</t>
@@ -376,6 +391,9 @@
   </si>
   <si>
     <t>Unusual</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -541,7 +559,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="26">
     <dxf>
       <font>
         <color rgb="FFD97706"/>
@@ -569,6 +587,16 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFDC2626"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEE2E2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -624,6 +652,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FFDC2626"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF047857"/>
       </font>
       <fill>
@@ -674,6 +712,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FFDC2626"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF047857"/>
       </font>
       <fill>
@@ -719,6 +767,16 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFDC2626"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEE2E2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1560,15 +1618,15 @@
         <v>0</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>40</v>
@@ -1592,18 +1650,18 @@
         <v>0</v>
       </c>
       <c r="J11" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D12" s="13">
         <v>0</v>
@@ -1618,24 +1676,24 @@
         <v>35000</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I12" s="13">
         <v>0</v>
       </c>
       <c r="J12" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D13" s="13">
         <v>0</v>
@@ -1650,24 +1708,24 @@
         <v>10000</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I13" s="13">
         <v>0</v>
       </c>
       <c r="J13" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D14" s="13">
         <v>0</v>
@@ -1682,24 +1740,24 @@
         <v>55000</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I14" s="13">
         <v>0</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D15" s="13">
         <v>0</v>
@@ -1714,24 +1772,24 @@
         <v>95000</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I15" s="13">
         <v>0</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D16" s="13">
         <v>0</v>
@@ -1746,24 +1804,24 @@
         <v>180000</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I16" s="13">
         <v>-2000</v>
       </c>
       <c r="J16" s="12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D17" s="13">
         <v>100000</v>
@@ -1778,24 +1836,24 @@
         <v>0</v>
       </c>
       <c r="H17" s="12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I17" s="13">
         <v>0</v>
       </c>
       <c r="J17" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D18" s="13">
         <v>60000</v>
@@ -1810,24 +1868,24 @@
         <v>0</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I18" s="13">
         <v>0</v>
       </c>
       <c r="J18" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D19" s="13">
         <v>20000</v>
@@ -1842,24 +1900,24 @@
         <v>0</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I19" s="13">
         <v>0</v>
       </c>
       <c r="J19" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D20" s="13">
         <v>5000</v>
@@ -1874,13 +1932,13 @@
         <v>0</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="I20" s="13">
         <v>0</v>
       </c>
       <c r="J20" s="12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -2917,10 +2975,10 @@
       <formula1>'Lists'!$A$2:$A$7</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="H10:H105">
-      <formula1>'Lists'!$B$2:$B$11</formula1>
+      <formula1>'Lists'!$B$2:$B$12</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="H6:H105">
-      <formula1>'Lists'!$B$2:$B$11</formula1>
+      <formula1>'Lists'!$B$2:$B$12</formula1>
     </dataValidation>
   </dataValidations>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -2945,7 +3003,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3173,15 +3231,15 @@
         <v>0</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>40</v>
@@ -3205,18 +3263,18 @@
         <v>0</v>
       </c>
       <c r="J11" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D12" s="13">
         <v>0</v>
@@ -3231,24 +3289,24 @@
         <v>35000</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I12" s="13">
         <v>0</v>
       </c>
       <c r="J12" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D13" s="13">
         <v>0</v>
@@ -3263,24 +3321,24 @@
         <v>10000</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I13" s="13">
         <v>0</v>
       </c>
       <c r="J13" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D14" s="13">
         <v>0</v>
@@ -3295,24 +3353,24 @@
         <v>55000</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I14" s="13">
         <v>0</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D15" s="13">
         <v>0</v>
@@ -3327,24 +3385,24 @@
         <v>95000</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I15" s="13">
         <v>0</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D16" s="13">
         <v>0</v>
@@ -3359,24 +3417,24 @@
         <v>180000</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I16" s="13">
         <v>-2000</v>
       </c>
       <c r="J16" s="12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D17" s="13">
         <v>100000</v>
@@ -3391,24 +3449,24 @@
         <v>0</v>
       </c>
       <c r="H17" s="12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I17" s="13">
         <v>0</v>
       </c>
       <c r="J17" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D18" s="13">
         <v>60000</v>
@@ -3423,24 +3481,24 @@
         <v>0</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I18" s="13">
         <v>0</v>
       </c>
       <c r="J18" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D19" s="13">
         <v>20000</v>
@@ -3455,24 +3513,24 @@
         <v>0</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I19" s="13">
         <v>0</v>
       </c>
       <c r="J19" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D20" s="13">
         <v>5000</v>
@@ -3487,13 +3545,13 @@
         <v>0</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="I20" s="13">
         <v>0</v>
       </c>
       <c r="J20" s="12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -4530,10 +4588,10 @@
       <formula1>'Lists'!$A$2:$A$7</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="H10:H105">
-      <formula1>'Lists'!$B$2:$B$11</formula1>
+      <formula1>'Lists'!$B$2:$B$12</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="H6:H105">
-      <formula1>'Lists'!$B$2:$B$11</formula1>
+      <formula1>'Lists'!$B$2:$B$12</formula1>
     </dataValidation>
   </dataValidations>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -4563,7 +4621,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4608,7 +4666,7 @@
     <row r="3" spans="1:19" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -4652,16 +4710,16 @@
         <v>34</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L5" s="10" t="s">
         <v>35</v>
@@ -4670,19 +4728,19 @@
         <v>36</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="Q5" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="S5" s="10" t="s">
         <v>37</v>
@@ -4746,7 +4804,7 @@
         <v>100000</v>
       </c>
       <c r="O6" s="14" t="str">
-        <f>IF(B6="","",IF(OR(C6="",L6=""),"Unmapped","OK"))</f>
+        <f>IF(B6="","",IF(L6="Unresolved","Unresolved",IF(OR(C6="",L6=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P6" s="14" t="str">
@@ -4758,7 +4816,7 @@
         <v>Review</v>
       </c>
       <c r="R6" s="14" t="str">
-        <f>IF(B6="","",IF(OR(O6&lt;&gt;"OK",P6&lt;&gt;"OK",Q6&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B6="","",IF(O6="Unresolved","Unresolved",IF(OR(O6&lt;&gt;"OK",P6&lt;&gt;"OK",Q6&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Review</v>
       </c>
       <c r="S6" s="14" t="str">
@@ -4824,7 +4882,7 @@
         <v>52000</v>
       </c>
       <c r="O7" s="14" t="str">
-        <f>IF(B7="","",IF(OR(C7="",L7=""),"Unmapped","OK"))</f>
+        <f>IF(B7="","",IF(L7="Unresolved","Unresolved",IF(OR(C7="",L7=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P7" s="14" t="str">
@@ -4836,7 +4894,7 @@
         <v>OK</v>
       </c>
       <c r="R7" s="14" t="str">
-        <f>IF(B7="","",IF(OR(O7&lt;&gt;"OK",P7&lt;&gt;"OK",Q7&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B7="","",IF(O7="Unresolved","Unresolved",IF(OR(O7&lt;&gt;"OK",P7&lt;&gt;"OK",Q7&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Complete</v>
       </c>
       <c r="S7" s="14" t="str">
@@ -4902,7 +4960,7 @@
         <v>30000</v>
       </c>
       <c r="O8" s="14" t="str">
-        <f>IF(B8="","",IF(OR(C8="",L8=""),"Unmapped","OK"))</f>
+        <f>IF(B8="","",IF(L8="Unresolved","Unresolved",IF(OR(C8="",L8=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P8" s="14" t="str">
@@ -4914,7 +4972,7 @@
         <v>Review</v>
       </c>
       <c r="R8" s="14" t="str">
-        <f>IF(B8="","",IF(OR(O8&lt;&gt;"OK",P8&lt;&gt;"OK",Q8&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B8="","",IF(O8="Unresolved","Unresolved",IF(OR(O8&lt;&gt;"OK",P8&lt;&gt;"OK",Q8&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Review</v>
       </c>
       <c r="S8" s="14" t="str">
@@ -4969,7 +5027,7 @@
       </c>
       <c r="L9" s="14" t="str">
         <f>IF('Start Here'!$B$8="Paste Import",'Paste Import'!H9,'Manual Input'!H9)</f>
-        <v>Other</v>
+        <v>Unresolved</v>
       </c>
       <c r="M9" s="15">
         <f>IF('Start Here'!$B$8="Paste Import",'Paste Import'!I9,'Manual Input'!I9)</f>
@@ -4980,8 +5038,8 @@
         <v>5000</v>
       </c>
       <c r="O9" s="14" t="str">
-        <f>IF(B9="","",IF(OR(C9="",L9=""),"Unmapped","OK"))</f>
-        <v>OK</v>
+        <f>IF(B9="","",IF(L9="Unresolved","Unresolved",IF(OR(C9="",L9=""),"Unmapped","OK")))</f>
+        <v>Unresolved</v>
       </c>
       <c r="P9" s="14" t="str">
         <f>IF(B9="","",IF(OR(AND(OR(C9="Asset",C9="Expense"),H9&lt;0),AND(OR(C9="Liability",C9="Equity",C9="Revenue"),H9&gt;0)),"Unusual","OK"))</f>
@@ -4992,12 +5050,12 @@
         <v>OK</v>
       </c>
       <c r="R9" s="14" t="str">
-        <f>IF(B9="","",IF(OR(O9&lt;&gt;"OK",P9&lt;&gt;"OK",Q9&lt;&gt;"OK"),"Review","Complete"))</f>
-        <v>Complete</v>
+        <f>IF(B9="","",IF(O9="Unresolved","Unresolved",IF(OR(O9&lt;&gt;"OK",P9&lt;&gt;"OK",Q9&lt;&gt;"OK"),"Review","Complete")))</f>
+        <v>Unresolved</v>
       </c>
       <c r="S9" s="14" t="str">
         <f>IF('Start Here'!$B$8="Paste Import",'Paste Import'!J9,'Manual Input'!J9)</f>
-        <v/>
+        <v>Classification support is unresolved</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -5058,7 +5116,7 @@
         <v>80000</v>
       </c>
       <c r="O10" s="14" t="str">
-        <f>IF(B10="","",IF(OR(C10="",L10=""),"Unmapped","OK"))</f>
+        <f>IF(B10="","",IF(L10="Unresolved","Unresolved",IF(OR(C10="",L10=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P10" s="14" t="str">
@@ -5070,7 +5128,7 @@
         <v>OK</v>
       </c>
       <c r="R10" s="14" t="str">
-        <f>IF(B10="","",IF(OR(O10&lt;&gt;"OK",P10&lt;&gt;"OK",Q10&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B10="","",IF(O10="Unresolved","Unresolved",IF(OR(O10&lt;&gt;"OK",P10&lt;&gt;"OK",Q10&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Complete</v>
       </c>
       <c r="S10" s="14" t="str">
@@ -5136,7 +5194,7 @@
         <v>-25000</v>
       </c>
       <c r="O11" s="14" t="str">
-        <f>IF(B11="","",IF(OR(C11="",L11=""),"Unmapped","OK"))</f>
+        <f>IF(B11="","",IF(L11="Unresolved","Unresolved",IF(OR(C11="",L11=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P11" s="14" t="str">
@@ -5148,7 +5206,7 @@
         <v>Review</v>
       </c>
       <c r="R11" s="14" t="str">
-        <f>IF(B11="","",IF(OR(O11&lt;&gt;"OK",P11&lt;&gt;"OK",Q11&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B11="","",IF(O11="Unresolved","Unresolved",IF(OR(O11&lt;&gt;"OK",P11&lt;&gt;"OK",Q11&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Review</v>
       </c>
       <c r="S11" s="14" t="str">
@@ -5214,7 +5272,7 @@
         <v>-40000</v>
       </c>
       <c r="O12" s="14" t="str">
-        <f>IF(B12="","",IF(OR(C12="",L12=""),"Unmapped","OK"))</f>
+        <f>IF(B12="","",IF(L12="Unresolved","Unresolved",IF(OR(C12="",L12=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P12" s="14" t="str">
@@ -5226,7 +5284,7 @@
         <v>Review</v>
       </c>
       <c r="R12" s="14" t="str">
-        <f>IF(B12="","",IF(OR(O12&lt;&gt;"OK",P12&lt;&gt;"OK",Q12&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B12="","",IF(O12="Unresolved","Unresolved",IF(OR(O12&lt;&gt;"OK",P12&lt;&gt;"OK",Q12&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Review</v>
       </c>
       <c r="S12" s="14" t="str">
@@ -5292,7 +5350,7 @@
         <v>-15000</v>
       </c>
       <c r="O13" s="14" t="str">
-        <f>IF(B13="","",IF(OR(C13="",L13=""),"Unmapped","OK"))</f>
+        <f>IF(B13="","",IF(L13="Unresolved","Unresolved",IF(OR(C13="",L13=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P13" s="14" t="str">
@@ -5304,7 +5362,7 @@
         <v>Review</v>
       </c>
       <c r="R13" s="14" t="str">
-        <f>IF(B13="","",IF(OR(O13&lt;&gt;"OK",P13&lt;&gt;"OK",Q13&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B13="","",IF(O13="Unresolved","Unresolved",IF(OR(O13&lt;&gt;"OK",P13&lt;&gt;"OK",Q13&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Review</v>
       </c>
       <c r="S13" s="14" t="str">
@@ -5370,7 +5428,7 @@
         <v>-60000</v>
       </c>
       <c r="O14" s="14" t="str">
-        <f>IF(B14="","",IF(OR(C14="",L14=""),"Unmapped","OK"))</f>
+        <f>IF(B14="","",IF(L14="Unresolved","Unresolved",IF(OR(C14="",L14=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P14" s="14" t="str">
@@ -5382,7 +5440,7 @@
         <v>OK</v>
       </c>
       <c r="R14" s="14" t="str">
-        <f>IF(B14="","",IF(OR(O14&lt;&gt;"OK",P14&lt;&gt;"OK",Q14&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B14="","",IF(O14="Unresolved","Unresolved",IF(OR(O14&lt;&gt;"OK",P14&lt;&gt;"OK",Q14&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Complete</v>
       </c>
       <c r="S14" s="14" t="str">
@@ -5448,7 +5506,7 @@
         <v>-110000</v>
       </c>
       <c r="O15" s="14" t="str">
-        <f>IF(B15="","",IF(OR(C15="",L15=""),"Unmapped","OK"))</f>
+        <f>IF(B15="","",IF(L15="Unresolved","Unresolved",IF(OR(C15="",L15=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P15" s="14" t="str">
@@ -5460,7 +5518,7 @@
         <v>Review</v>
       </c>
       <c r="R15" s="14" t="str">
-        <f>IF(B15="","",IF(OR(O15&lt;&gt;"OK",P15&lt;&gt;"OK",Q15&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B15="","",IF(O15="Unresolved","Unresolved",IF(OR(O15&lt;&gt;"OK",P15&lt;&gt;"OK",Q15&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Review</v>
       </c>
       <c r="S15" s="14" t="str">
@@ -5526,7 +5584,7 @@
         <v>-202000</v>
       </c>
       <c r="O16" s="14" t="str">
-        <f>IF(B16="","",IF(OR(C16="",L16=""),"Unmapped","OK"))</f>
+        <f>IF(B16="","",IF(L16="Unresolved","Unresolved",IF(OR(C16="",L16=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P16" s="14" t="str">
@@ -5538,7 +5596,7 @@
         <v>Review</v>
       </c>
       <c r="R16" s="14" t="str">
-        <f>IF(B16="","",IF(OR(O16&lt;&gt;"OK",P16&lt;&gt;"OK",Q16&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B16="","",IF(O16="Unresolved","Unresolved",IF(OR(O16&lt;&gt;"OK",P16&lt;&gt;"OK",Q16&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Review</v>
       </c>
       <c r="S16" s="14" t="str">
@@ -5604,7 +5662,7 @@
         <v>100000</v>
       </c>
       <c r="O17" s="14" t="str">
-        <f>IF(B17="","",IF(OR(C17="",L17=""),"Unmapped","OK"))</f>
+        <f>IF(B17="","",IF(L17="Unresolved","Unresolved",IF(OR(C17="",L17=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P17" s="14" t="str">
@@ -5616,7 +5674,7 @@
         <v>Review</v>
       </c>
       <c r="R17" s="14" t="str">
-        <f>IF(B17="","",IF(OR(O17&lt;&gt;"OK",P17&lt;&gt;"OK",Q17&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B17="","",IF(O17="Unresolved","Unresolved",IF(OR(O17&lt;&gt;"OK",P17&lt;&gt;"OK",Q17&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Review</v>
       </c>
       <c r="S17" s="14" t="str">
@@ -5682,7 +5740,7 @@
         <v>60000</v>
       </c>
       <c r="O18" s="14" t="str">
-        <f>IF(B18="","",IF(OR(C18="",L18=""),"Unmapped","OK"))</f>
+        <f>IF(B18="","",IF(L18="Unresolved","Unresolved",IF(OR(C18="",L18=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P18" s="14" t="str">
@@ -5694,7 +5752,7 @@
         <v>OK</v>
       </c>
       <c r="R18" s="14" t="str">
-        <f>IF(B18="","",IF(OR(O18&lt;&gt;"OK",P18&lt;&gt;"OK",Q18&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B18="","",IF(O18="Unresolved","Unresolved",IF(OR(O18&lt;&gt;"OK",P18&lt;&gt;"OK",Q18&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Complete</v>
       </c>
       <c r="S18" s="14" t="str">
@@ -5760,7 +5818,7 @@
         <v>20000</v>
       </c>
       <c r="O19" s="14" t="str">
-        <f>IF(B19="","",IF(OR(C19="",L19=""),"Unmapped","OK"))</f>
+        <f>IF(B19="","",IF(L19="Unresolved","Unresolved",IF(OR(C19="",L19=""),"Unmapped","OK")))</f>
         <v>OK</v>
       </c>
       <c r="P19" s="14" t="str">
@@ -5772,7 +5830,7 @@
         <v>OK</v>
       </c>
       <c r="R19" s="14" t="str">
-        <f>IF(B19="","",IF(OR(O19&lt;&gt;"OK",P19&lt;&gt;"OK",Q19&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B19="","",IF(O19="Unresolved","Unresolved",IF(OR(O19&lt;&gt;"OK",P19&lt;&gt;"OK",Q19&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Complete</v>
       </c>
       <c r="S19" s="14" t="str">
@@ -5838,7 +5896,7 @@
         <v>5000</v>
       </c>
       <c r="O20" s="14" t="str">
-        <f>IF(B20="","",IF(OR(C20="",L20=""),"Unmapped","OK"))</f>
+        <f>IF(B20="","",IF(L20="Unresolved","Unresolved",IF(OR(C20="",L20=""),"Unmapped","OK")))</f>
         <v>Unmapped</v>
       </c>
       <c r="P20" s="14" t="str">
@@ -5850,7 +5908,7 @@
         <v>Review</v>
       </c>
       <c r="R20" s="14" t="str">
-        <f>IF(B20="","",IF(OR(O20&lt;&gt;"OK",P20&lt;&gt;"OK",Q20&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B20="","",IF(O20="Unresolved","Unresolved",IF(OR(O20&lt;&gt;"OK",P20&lt;&gt;"OK",Q20&lt;&gt;"OK"),"Review","Complete")))</f>
         <v>Review</v>
       </c>
       <c r="S20" s="14" t="str">
@@ -5916,7 +5974,7 @@
         <v/>
       </c>
       <c r="O21" s="14" t="str">
-        <f>IF(B21="","",IF(OR(C21="",L21=""),"Unmapped","OK"))</f>
+        <f>IF(B21="","",IF(L21="Unresolved","Unresolved",IF(OR(C21="",L21=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P21" s="14" t="str">
@@ -5928,7 +5986,7 @@
         <v/>
       </c>
       <c r="R21" s="14" t="str">
-        <f>IF(B21="","",IF(OR(O21&lt;&gt;"OK",P21&lt;&gt;"OK",Q21&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B21="","",IF(O21="Unresolved","Unresolved",IF(OR(O21&lt;&gt;"OK",P21&lt;&gt;"OK",Q21&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S21" s="14" t="str">
@@ -5994,7 +6052,7 @@
         <v/>
       </c>
       <c r="O22" s="14" t="str">
-        <f>IF(B22="","",IF(OR(C22="",L22=""),"Unmapped","OK"))</f>
+        <f>IF(B22="","",IF(L22="Unresolved","Unresolved",IF(OR(C22="",L22=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P22" s="14" t="str">
@@ -6006,7 +6064,7 @@
         <v/>
       </c>
       <c r="R22" s="14" t="str">
-        <f>IF(B22="","",IF(OR(O22&lt;&gt;"OK",P22&lt;&gt;"OK",Q22&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B22="","",IF(O22="Unresolved","Unresolved",IF(OR(O22&lt;&gt;"OK",P22&lt;&gt;"OK",Q22&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S22" s="14" t="str">
@@ -6072,7 +6130,7 @@
         <v/>
       </c>
       <c r="O23" s="14" t="str">
-        <f>IF(B23="","",IF(OR(C23="",L23=""),"Unmapped","OK"))</f>
+        <f>IF(B23="","",IF(L23="Unresolved","Unresolved",IF(OR(C23="",L23=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P23" s="14" t="str">
@@ -6084,7 +6142,7 @@
         <v/>
       </c>
       <c r="R23" s="14" t="str">
-        <f>IF(B23="","",IF(OR(O23&lt;&gt;"OK",P23&lt;&gt;"OK",Q23&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B23="","",IF(O23="Unresolved","Unresolved",IF(OR(O23&lt;&gt;"OK",P23&lt;&gt;"OK",Q23&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S23" s="14" t="str">
@@ -6150,7 +6208,7 @@
         <v/>
       </c>
       <c r="O24" s="14" t="str">
-        <f>IF(B24="","",IF(OR(C24="",L24=""),"Unmapped","OK"))</f>
+        <f>IF(B24="","",IF(L24="Unresolved","Unresolved",IF(OR(C24="",L24=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P24" s="14" t="str">
@@ -6162,7 +6220,7 @@
         <v/>
       </c>
       <c r="R24" s="14" t="str">
-        <f>IF(B24="","",IF(OR(O24&lt;&gt;"OK",P24&lt;&gt;"OK",Q24&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B24="","",IF(O24="Unresolved","Unresolved",IF(OR(O24&lt;&gt;"OK",P24&lt;&gt;"OK",Q24&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S24" s="14" t="str">
@@ -6228,7 +6286,7 @@
         <v/>
       </c>
       <c r="O25" s="14" t="str">
-        <f>IF(B25="","",IF(OR(C25="",L25=""),"Unmapped","OK"))</f>
+        <f>IF(B25="","",IF(L25="Unresolved","Unresolved",IF(OR(C25="",L25=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P25" s="14" t="str">
@@ -6240,7 +6298,7 @@
         <v/>
       </c>
       <c r="R25" s="14" t="str">
-        <f>IF(B25="","",IF(OR(O25&lt;&gt;"OK",P25&lt;&gt;"OK",Q25&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B25="","",IF(O25="Unresolved","Unresolved",IF(OR(O25&lt;&gt;"OK",P25&lt;&gt;"OK",Q25&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S25" s="14" t="str">
@@ -6306,7 +6364,7 @@
         <v/>
       </c>
       <c r="O26" s="14" t="str">
-        <f>IF(B26="","",IF(OR(C26="",L26=""),"Unmapped","OK"))</f>
+        <f>IF(B26="","",IF(L26="Unresolved","Unresolved",IF(OR(C26="",L26=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P26" s="14" t="str">
@@ -6318,7 +6376,7 @@
         <v/>
       </c>
       <c r="R26" s="14" t="str">
-        <f>IF(B26="","",IF(OR(O26&lt;&gt;"OK",P26&lt;&gt;"OK",Q26&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B26="","",IF(O26="Unresolved","Unresolved",IF(OR(O26&lt;&gt;"OK",P26&lt;&gt;"OK",Q26&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S26" s="14" t="str">
@@ -6384,7 +6442,7 @@
         <v/>
       </c>
       <c r="O27" s="14" t="str">
-        <f>IF(B27="","",IF(OR(C27="",L27=""),"Unmapped","OK"))</f>
+        <f>IF(B27="","",IF(L27="Unresolved","Unresolved",IF(OR(C27="",L27=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P27" s="14" t="str">
@@ -6396,7 +6454,7 @@
         <v/>
       </c>
       <c r="R27" s="14" t="str">
-        <f>IF(B27="","",IF(OR(O27&lt;&gt;"OK",P27&lt;&gt;"OK",Q27&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B27="","",IF(O27="Unresolved","Unresolved",IF(OR(O27&lt;&gt;"OK",P27&lt;&gt;"OK",Q27&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S27" s="14" t="str">
@@ -6462,7 +6520,7 @@
         <v/>
       </c>
       <c r="O28" s="14" t="str">
-        <f>IF(B28="","",IF(OR(C28="",L28=""),"Unmapped","OK"))</f>
+        <f>IF(B28="","",IF(L28="Unresolved","Unresolved",IF(OR(C28="",L28=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P28" s="14" t="str">
@@ -6474,7 +6532,7 @@
         <v/>
       </c>
       <c r="R28" s="14" t="str">
-        <f>IF(B28="","",IF(OR(O28&lt;&gt;"OK",P28&lt;&gt;"OK",Q28&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B28="","",IF(O28="Unresolved","Unresolved",IF(OR(O28&lt;&gt;"OK",P28&lt;&gt;"OK",Q28&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S28" s="14" t="str">
@@ -6540,7 +6598,7 @@
         <v/>
       </c>
       <c r="O29" s="14" t="str">
-        <f>IF(B29="","",IF(OR(C29="",L29=""),"Unmapped","OK"))</f>
+        <f>IF(B29="","",IF(L29="Unresolved","Unresolved",IF(OR(C29="",L29=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P29" s="14" t="str">
@@ -6552,7 +6610,7 @@
         <v/>
       </c>
       <c r="R29" s="14" t="str">
-        <f>IF(B29="","",IF(OR(O29&lt;&gt;"OK",P29&lt;&gt;"OK",Q29&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B29="","",IF(O29="Unresolved","Unresolved",IF(OR(O29&lt;&gt;"OK",P29&lt;&gt;"OK",Q29&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S29" s="14" t="str">
@@ -6618,7 +6676,7 @@
         <v/>
       </c>
       <c r="O30" s="14" t="str">
-        <f>IF(B30="","",IF(OR(C30="",L30=""),"Unmapped","OK"))</f>
+        <f>IF(B30="","",IF(L30="Unresolved","Unresolved",IF(OR(C30="",L30=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P30" s="14" t="str">
@@ -6630,7 +6688,7 @@
         <v/>
       </c>
       <c r="R30" s="14" t="str">
-        <f>IF(B30="","",IF(OR(O30&lt;&gt;"OK",P30&lt;&gt;"OK",Q30&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B30="","",IF(O30="Unresolved","Unresolved",IF(OR(O30&lt;&gt;"OK",P30&lt;&gt;"OK",Q30&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S30" s="14" t="str">
@@ -6696,7 +6754,7 @@
         <v/>
       </c>
       <c r="O31" s="14" t="str">
-        <f>IF(B31="","",IF(OR(C31="",L31=""),"Unmapped","OK"))</f>
+        <f>IF(B31="","",IF(L31="Unresolved","Unresolved",IF(OR(C31="",L31=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P31" s="14" t="str">
@@ -6708,7 +6766,7 @@
         <v/>
       </c>
       <c r="R31" s="14" t="str">
-        <f>IF(B31="","",IF(OR(O31&lt;&gt;"OK",P31&lt;&gt;"OK",Q31&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B31="","",IF(O31="Unresolved","Unresolved",IF(OR(O31&lt;&gt;"OK",P31&lt;&gt;"OK",Q31&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S31" s="14" t="str">
@@ -6774,7 +6832,7 @@
         <v/>
       </c>
       <c r="O32" s="14" t="str">
-        <f>IF(B32="","",IF(OR(C32="",L32=""),"Unmapped","OK"))</f>
+        <f>IF(B32="","",IF(L32="Unresolved","Unresolved",IF(OR(C32="",L32=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P32" s="14" t="str">
@@ -6786,7 +6844,7 @@
         <v/>
       </c>
       <c r="R32" s="14" t="str">
-        <f>IF(B32="","",IF(OR(O32&lt;&gt;"OK",P32&lt;&gt;"OK",Q32&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B32="","",IF(O32="Unresolved","Unresolved",IF(OR(O32&lt;&gt;"OK",P32&lt;&gt;"OK",Q32&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S32" s="14" t="str">
@@ -6852,7 +6910,7 @@
         <v/>
       </c>
       <c r="O33" s="14" t="str">
-        <f>IF(B33="","",IF(OR(C33="",L33=""),"Unmapped","OK"))</f>
+        <f>IF(B33="","",IF(L33="Unresolved","Unresolved",IF(OR(C33="",L33=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P33" s="14" t="str">
@@ -6864,7 +6922,7 @@
         <v/>
       </c>
       <c r="R33" s="14" t="str">
-        <f>IF(B33="","",IF(OR(O33&lt;&gt;"OK",P33&lt;&gt;"OK",Q33&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B33="","",IF(O33="Unresolved","Unresolved",IF(OR(O33&lt;&gt;"OK",P33&lt;&gt;"OK",Q33&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S33" s="14" t="str">
@@ -6930,7 +6988,7 @@
         <v/>
       </c>
       <c r="O34" s="14" t="str">
-        <f>IF(B34="","",IF(OR(C34="",L34=""),"Unmapped","OK"))</f>
+        <f>IF(B34="","",IF(L34="Unresolved","Unresolved",IF(OR(C34="",L34=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P34" s="14" t="str">
@@ -6942,7 +7000,7 @@
         <v/>
       </c>
       <c r="R34" s="14" t="str">
-        <f>IF(B34="","",IF(OR(O34&lt;&gt;"OK",P34&lt;&gt;"OK",Q34&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B34="","",IF(O34="Unresolved","Unresolved",IF(OR(O34&lt;&gt;"OK",P34&lt;&gt;"OK",Q34&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S34" s="14" t="str">
@@ -7008,7 +7066,7 @@
         <v/>
       </c>
       <c r="O35" s="14" t="str">
-        <f>IF(B35="","",IF(OR(C35="",L35=""),"Unmapped","OK"))</f>
+        <f>IF(B35="","",IF(L35="Unresolved","Unresolved",IF(OR(C35="",L35=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P35" s="14" t="str">
@@ -7020,7 +7078,7 @@
         <v/>
       </c>
       <c r="R35" s="14" t="str">
-        <f>IF(B35="","",IF(OR(O35&lt;&gt;"OK",P35&lt;&gt;"OK",Q35&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B35="","",IF(O35="Unresolved","Unresolved",IF(OR(O35&lt;&gt;"OK",P35&lt;&gt;"OK",Q35&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S35" s="14" t="str">
@@ -7086,7 +7144,7 @@
         <v/>
       </c>
       <c r="O36" s="14" t="str">
-        <f>IF(B36="","",IF(OR(C36="",L36=""),"Unmapped","OK"))</f>
+        <f>IF(B36="","",IF(L36="Unresolved","Unresolved",IF(OR(C36="",L36=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P36" s="14" t="str">
@@ -7098,7 +7156,7 @@
         <v/>
       </c>
       <c r="R36" s="14" t="str">
-        <f>IF(B36="","",IF(OR(O36&lt;&gt;"OK",P36&lt;&gt;"OK",Q36&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B36="","",IF(O36="Unresolved","Unresolved",IF(OR(O36&lt;&gt;"OK",P36&lt;&gt;"OK",Q36&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S36" s="14" t="str">
@@ -7164,7 +7222,7 @@
         <v/>
       </c>
       <c r="O37" s="14" t="str">
-        <f>IF(B37="","",IF(OR(C37="",L37=""),"Unmapped","OK"))</f>
+        <f>IF(B37="","",IF(L37="Unresolved","Unresolved",IF(OR(C37="",L37=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P37" s="14" t="str">
@@ -7176,7 +7234,7 @@
         <v/>
       </c>
       <c r="R37" s="14" t="str">
-        <f>IF(B37="","",IF(OR(O37&lt;&gt;"OK",P37&lt;&gt;"OK",Q37&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B37="","",IF(O37="Unresolved","Unresolved",IF(OR(O37&lt;&gt;"OK",P37&lt;&gt;"OK",Q37&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S37" s="14" t="str">
@@ -7242,7 +7300,7 @@
         <v/>
       </c>
       <c r="O38" s="14" t="str">
-        <f>IF(B38="","",IF(OR(C38="",L38=""),"Unmapped","OK"))</f>
+        <f>IF(B38="","",IF(L38="Unresolved","Unresolved",IF(OR(C38="",L38=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P38" s="14" t="str">
@@ -7254,7 +7312,7 @@
         <v/>
       </c>
       <c r="R38" s="14" t="str">
-        <f>IF(B38="","",IF(OR(O38&lt;&gt;"OK",P38&lt;&gt;"OK",Q38&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B38="","",IF(O38="Unresolved","Unresolved",IF(OR(O38&lt;&gt;"OK",P38&lt;&gt;"OK",Q38&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S38" s="14" t="str">
@@ -7320,7 +7378,7 @@
         <v/>
       </c>
       <c r="O39" s="14" t="str">
-        <f>IF(B39="","",IF(OR(C39="",L39=""),"Unmapped","OK"))</f>
+        <f>IF(B39="","",IF(L39="Unresolved","Unresolved",IF(OR(C39="",L39=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P39" s="14" t="str">
@@ -7332,7 +7390,7 @@
         <v/>
       </c>
       <c r="R39" s="14" t="str">
-        <f>IF(B39="","",IF(OR(O39&lt;&gt;"OK",P39&lt;&gt;"OK",Q39&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B39="","",IF(O39="Unresolved","Unresolved",IF(OR(O39&lt;&gt;"OK",P39&lt;&gt;"OK",Q39&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S39" s="14" t="str">
@@ -7398,7 +7456,7 @@
         <v/>
       </c>
       <c r="O40" s="14" t="str">
-        <f>IF(B40="","",IF(OR(C40="",L40=""),"Unmapped","OK"))</f>
+        <f>IF(B40="","",IF(L40="Unresolved","Unresolved",IF(OR(C40="",L40=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P40" s="14" t="str">
@@ -7410,7 +7468,7 @@
         <v/>
       </c>
       <c r="R40" s="14" t="str">
-        <f>IF(B40="","",IF(OR(O40&lt;&gt;"OK",P40&lt;&gt;"OK",Q40&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B40="","",IF(O40="Unresolved","Unresolved",IF(OR(O40&lt;&gt;"OK",P40&lt;&gt;"OK",Q40&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S40" s="14" t="str">
@@ -7476,7 +7534,7 @@
         <v/>
       </c>
       <c r="O41" s="14" t="str">
-        <f>IF(B41="","",IF(OR(C41="",L41=""),"Unmapped","OK"))</f>
+        <f>IF(B41="","",IF(L41="Unresolved","Unresolved",IF(OR(C41="",L41=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P41" s="14" t="str">
@@ -7488,7 +7546,7 @@
         <v/>
       </c>
       <c r="R41" s="14" t="str">
-        <f>IF(B41="","",IF(OR(O41&lt;&gt;"OK",P41&lt;&gt;"OK",Q41&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B41="","",IF(O41="Unresolved","Unresolved",IF(OR(O41&lt;&gt;"OK",P41&lt;&gt;"OK",Q41&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S41" s="14" t="str">
@@ -7554,7 +7612,7 @@
         <v/>
       </c>
       <c r="O42" s="14" t="str">
-        <f>IF(B42="","",IF(OR(C42="",L42=""),"Unmapped","OK"))</f>
+        <f>IF(B42="","",IF(L42="Unresolved","Unresolved",IF(OR(C42="",L42=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P42" s="14" t="str">
@@ -7566,7 +7624,7 @@
         <v/>
       </c>
       <c r="R42" s="14" t="str">
-        <f>IF(B42="","",IF(OR(O42&lt;&gt;"OK",P42&lt;&gt;"OK",Q42&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B42="","",IF(O42="Unresolved","Unresolved",IF(OR(O42&lt;&gt;"OK",P42&lt;&gt;"OK",Q42&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S42" s="14" t="str">
@@ -7632,7 +7690,7 @@
         <v/>
       </c>
       <c r="O43" s="14" t="str">
-        <f>IF(B43="","",IF(OR(C43="",L43=""),"Unmapped","OK"))</f>
+        <f>IF(B43="","",IF(L43="Unresolved","Unresolved",IF(OR(C43="",L43=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P43" s="14" t="str">
@@ -7644,7 +7702,7 @@
         <v/>
       </c>
       <c r="R43" s="14" t="str">
-        <f>IF(B43="","",IF(OR(O43&lt;&gt;"OK",P43&lt;&gt;"OK",Q43&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B43="","",IF(O43="Unresolved","Unresolved",IF(OR(O43&lt;&gt;"OK",P43&lt;&gt;"OK",Q43&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S43" s="14" t="str">
@@ -7710,7 +7768,7 @@
         <v/>
       </c>
       <c r="O44" s="14" t="str">
-        <f>IF(B44="","",IF(OR(C44="",L44=""),"Unmapped","OK"))</f>
+        <f>IF(B44="","",IF(L44="Unresolved","Unresolved",IF(OR(C44="",L44=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P44" s="14" t="str">
@@ -7722,7 +7780,7 @@
         <v/>
       </c>
       <c r="R44" s="14" t="str">
-        <f>IF(B44="","",IF(OR(O44&lt;&gt;"OK",P44&lt;&gt;"OK",Q44&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B44="","",IF(O44="Unresolved","Unresolved",IF(OR(O44&lt;&gt;"OK",P44&lt;&gt;"OK",Q44&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S44" s="14" t="str">
@@ -7788,7 +7846,7 @@
         <v/>
       </c>
       <c r="O45" s="14" t="str">
-        <f>IF(B45="","",IF(OR(C45="",L45=""),"Unmapped","OK"))</f>
+        <f>IF(B45="","",IF(L45="Unresolved","Unresolved",IF(OR(C45="",L45=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P45" s="14" t="str">
@@ -7800,7 +7858,7 @@
         <v/>
       </c>
       <c r="R45" s="14" t="str">
-        <f>IF(B45="","",IF(OR(O45&lt;&gt;"OK",P45&lt;&gt;"OK",Q45&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B45="","",IF(O45="Unresolved","Unresolved",IF(OR(O45&lt;&gt;"OK",P45&lt;&gt;"OK",Q45&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S45" s="14" t="str">
@@ -7866,7 +7924,7 @@
         <v/>
       </c>
       <c r="O46" s="14" t="str">
-        <f>IF(B46="","",IF(OR(C46="",L46=""),"Unmapped","OK"))</f>
+        <f>IF(B46="","",IF(L46="Unresolved","Unresolved",IF(OR(C46="",L46=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P46" s="14" t="str">
@@ -7878,7 +7936,7 @@
         <v/>
       </c>
       <c r="R46" s="14" t="str">
-        <f>IF(B46="","",IF(OR(O46&lt;&gt;"OK",P46&lt;&gt;"OK",Q46&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B46="","",IF(O46="Unresolved","Unresolved",IF(OR(O46&lt;&gt;"OK",P46&lt;&gt;"OK",Q46&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S46" s="14" t="str">
@@ -7944,7 +8002,7 @@
         <v/>
       </c>
       <c r="O47" s="14" t="str">
-        <f>IF(B47="","",IF(OR(C47="",L47=""),"Unmapped","OK"))</f>
+        <f>IF(B47="","",IF(L47="Unresolved","Unresolved",IF(OR(C47="",L47=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P47" s="14" t="str">
@@ -7956,7 +8014,7 @@
         <v/>
       </c>
       <c r="R47" s="14" t="str">
-        <f>IF(B47="","",IF(OR(O47&lt;&gt;"OK",P47&lt;&gt;"OK",Q47&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B47="","",IF(O47="Unresolved","Unresolved",IF(OR(O47&lt;&gt;"OK",P47&lt;&gt;"OK",Q47&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S47" s="14" t="str">
@@ -8022,7 +8080,7 @@
         <v/>
       </c>
       <c r="O48" s="14" t="str">
-        <f>IF(B48="","",IF(OR(C48="",L48=""),"Unmapped","OK"))</f>
+        <f>IF(B48="","",IF(L48="Unresolved","Unresolved",IF(OR(C48="",L48=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P48" s="14" t="str">
@@ -8034,7 +8092,7 @@
         <v/>
       </c>
       <c r="R48" s="14" t="str">
-        <f>IF(B48="","",IF(OR(O48&lt;&gt;"OK",P48&lt;&gt;"OK",Q48&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B48="","",IF(O48="Unresolved","Unresolved",IF(OR(O48&lt;&gt;"OK",P48&lt;&gt;"OK",Q48&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S48" s="14" t="str">
@@ -8100,7 +8158,7 @@
         <v/>
       </c>
       <c r="O49" s="14" t="str">
-        <f>IF(B49="","",IF(OR(C49="",L49=""),"Unmapped","OK"))</f>
+        <f>IF(B49="","",IF(L49="Unresolved","Unresolved",IF(OR(C49="",L49=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P49" s="14" t="str">
@@ -8112,7 +8170,7 @@
         <v/>
       </c>
       <c r="R49" s="14" t="str">
-        <f>IF(B49="","",IF(OR(O49&lt;&gt;"OK",P49&lt;&gt;"OK",Q49&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B49="","",IF(O49="Unresolved","Unresolved",IF(OR(O49&lt;&gt;"OK",P49&lt;&gt;"OK",Q49&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S49" s="14" t="str">
@@ -8178,7 +8236,7 @@
         <v/>
       </c>
       <c r="O50" s="14" t="str">
-        <f>IF(B50="","",IF(OR(C50="",L50=""),"Unmapped","OK"))</f>
+        <f>IF(B50="","",IF(L50="Unresolved","Unresolved",IF(OR(C50="",L50=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P50" s="14" t="str">
@@ -8190,7 +8248,7 @@
         <v/>
       </c>
       <c r="R50" s="14" t="str">
-        <f>IF(B50="","",IF(OR(O50&lt;&gt;"OK",P50&lt;&gt;"OK",Q50&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B50="","",IF(O50="Unresolved","Unresolved",IF(OR(O50&lt;&gt;"OK",P50&lt;&gt;"OK",Q50&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S50" s="14" t="str">
@@ -8256,7 +8314,7 @@
         <v/>
       </c>
       <c r="O51" s="14" t="str">
-        <f>IF(B51="","",IF(OR(C51="",L51=""),"Unmapped","OK"))</f>
+        <f>IF(B51="","",IF(L51="Unresolved","Unresolved",IF(OR(C51="",L51=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P51" s="14" t="str">
@@ -8268,7 +8326,7 @@
         <v/>
       </c>
       <c r="R51" s="14" t="str">
-        <f>IF(B51="","",IF(OR(O51&lt;&gt;"OK",P51&lt;&gt;"OK",Q51&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B51="","",IF(O51="Unresolved","Unresolved",IF(OR(O51&lt;&gt;"OK",P51&lt;&gt;"OK",Q51&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S51" s="14" t="str">
@@ -8334,7 +8392,7 @@
         <v/>
       </c>
       <c r="O52" s="14" t="str">
-        <f>IF(B52="","",IF(OR(C52="",L52=""),"Unmapped","OK"))</f>
+        <f>IF(B52="","",IF(L52="Unresolved","Unresolved",IF(OR(C52="",L52=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P52" s="14" t="str">
@@ -8346,7 +8404,7 @@
         <v/>
       </c>
       <c r="R52" s="14" t="str">
-        <f>IF(B52="","",IF(OR(O52&lt;&gt;"OK",P52&lt;&gt;"OK",Q52&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B52="","",IF(O52="Unresolved","Unresolved",IF(OR(O52&lt;&gt;"OK",P52&lt;&gt;"OK",Q52&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S52" s="14" t="str">
@@ -8412,7 +8470,7 @@
         <v/>
       </c>
       <c r="O53" s="14" t="str">
-        <f>IF(B53="","",IF(OR(C53="",L53=""),"Unmapped","OK"))</f>
+        <f>IF(B53="","",IF(L53="Unresolved","Unresolved",IF(OR(C53="",L53=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P53" s="14" t="str">
@@ -8424,7 +8482,7 @@
         <v/>
       </c>
       <c r="R53" s="14" t="str">
-        <f>IF(B53="","",IF(OR(O53&lt;&gt;"OK",P53&lt;&gt;"OK",Q53&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B53="","",IF(O53="Unresolved","Unresolved",IF(OR(O53&lt;&gt;"OK",P53&lt;&gt;"OK",Q53&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S53" s="14" t="str">
@@ -8490,7 +8548,7 @@
         <v/>
       </c>
       <c r="O54" s="14" t="str">
-        <f>IF(B54="","",IF(OR(C54="",L54=""),"Unmapped","OK"))</f>
+        <f>IF(B54="","",IF(L54="Unresolved","Unresolved",IF(OR(C54="",L54=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P54" s="14" t="str">
@@ -8502,7 +8560,7 @@
         <v/>
       </c>
       <c r="R54" s="14" t="str">
-        <f>IF(B54="","",IF(OR(O54&lt;&gt;"OK",P54&lt;&gt;"OK",Q54&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B54="","",IF(O54="Unresolved","Unresolved",IF(OR(O54&lt;&gt;"OK",P54&lt;&gt;"OK",Q54&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S54" s="14" t="str">
@@ -8568,7 +8626,7 @@
         <v/>
       </c>
       <c r="O55" s="14" t="str">
-        <f>IF(B55="","",IF(OR(C55="",L55=""),"Unmapped","OK"))</f>
+        <f>IF(B55="","",IF(L55="Unresolved","Unresolved",IF(OR(C55="",L55=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P55" s="14" t="str">
@@ -8580,7 +8638,7 @@
         <v/>
       </c>
       <c r="R55" s="14" t="str">
-        <f>IF(B55="","",IF(OR(O55&lt;&gt;"OK",P55&lt;&gt;"OK",Q55&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B55="","",IF(O55="Unresolved","Unresolved",IF(OR(O55&lt;&gt;"OK",P55&lt;&gt;"OK",Q55&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S55" s="14" t="str">
@@ -8646,7 +8704,7 @@
         <v/>
       </c>
       <c r="O56" s="14" t="str">
-        <f>IF(B56="","",IF(OR(C56="",L56=""),"Unmapped","OK"))</f>
+        <f>IF(B56="","",IF(L56="Unresolved","Unresolved",IF(OR(C56="",L56=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P56" s="14" t="str">
@@ -8658,7 +8716,7 @@
         <v/>
       </c>
       <c r="R56" s="14" t="str">
-        <f>IF(B56="","",IF(OR(O56&lt;&gt;"OK",P56&lt;&gt;"OK",Q56&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B56="","",IF(O56="Unresolved","Unresolved",IF(OR(O56&lt;&gt;"OK",P56&lt;&gt;"OK",Q56&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S56" s="14" t="str">
@@ -8724,7 +8782,7 @@
         <v/>
       </c>
       <c r="O57" s="14" t="str">
-        <f>IF(B57="","",IF(OR(C57="",L57=""),"Unmapped","OK"))</f>
+        <f>IF(B57="","",IF(L57="Unresolved","Unresolved",IF(OR(C57="",L57=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P57" s="14" t="str">
@@ -8736,7 +8794,7 @@
         <v/>
       </c>
       <c r="R57" s="14" t="str">
-        <f>IF(B57="","",IF(OR(O57&lt;&gt;"OK",P57&lt;&gt;"OK",Q57&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B57="","",IF(O57="Unresolved","Unresolved",IF(OR(O57&lt;&gt;"OK",P57&lt;&gt;"OK",Q57&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S57" s="14" t="str">
@@ -8802,7 +8860,7 @@
         <v/>
       </c>
       <c r="O58" s="14" t="str">
-        <f>IF(B58="","",IF(OR(C58="",L58=""),"Unmapped","OK"))</f>
+        <f>IF(B58="","",IF(L58="Unresolved","Unresolved",IF(OR(C58="",L58=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P58" s="14" t="str">
@@ -8814,7 +8872,7 @@
         <v/>
       </c>
       <c r="R58" s="14" t="str">
-        <f>IF(B58="","",IF(OR(O58&lt;&gt;"OK",P58&lt;&gt;"OK",Q58&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B58="","",IF(O58="Unresolved","Unresolved",IF(OR(O58&lt;&gt;"OK",P58&lt;&gt;"OK",Q58&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S58" s="14" t="str">
@@ -8880,7 +8938,7 @@
         <v/>
       </c>
       <c r="O59" s="14" t="str">
-        <f>IF(B59="","",IF(OR(C59="",L59=""),"Unmapped","OK"))</f>
+        <f>IF(B59="","",IF(L59="Unresolved","Unresolved",IF(OR(C59="",L59=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P59" s="14" t="str">
@@ -8892,7 +8950,7 @@
         <v/>
       </c>
       <c r="R59" s="14" t="str">
-        <f>IF(B59="","",IF(OR(O59&lt;&gt;"OK",P59&lt;&gt;"OK",Q59&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B59="","",IF(O59="Unresolved","Unresolved",IF(OR(O59&lt;&gt;"OK",P59&lt;&gt;"OK",Q59&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S59" s="14" t="str">
@@ -8958,7 +9016,7 @@
         <v/>
       </c>
       <c r="O60" s="14" t="str">
-        <f>IF(B60="","",IF(OR(C60="",L60=""),"Unmapped","OK"))</f>
+        <f>IF(B60="","",IF(L60="Unresolved","Unresolved",IF(OR(C60="",L60=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P60" s="14" t="str">
@@ -8970,7 +9028,7 @@
         <v/>
       </c>
       <c r="R60" s="14" t="str">
-        <f>IF(B60="","",IF(OR(O60&lt;&gt;"OK",P60&lt;&gt;"OK",Q60&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B60="","",IF(O60="Unresolved","Unresolved",IF(OR(O60&lt;&gt;"OK",P60&lt;&gt;"OK",Q60&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S60" s="14" t="str">
@@ -9036,7 +9094,7 @@
         <v/>
       </c>
       <c r="O61" s="14" t="str">
-        <f>IF(B61="","",IF(OR(C61="",L61=""),"Unmapped","OK"))</f>
+        <f>IF(B61="","",IF(L61="Unresolved","Unresolved",IF(OR(C61="",L61=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P61" s="14" t="str">
@@ -9048,7 +9106,7 @@
         <v/>
       </c>
       <c r="R61" s="14" t="str">
-        <f>IF(B61="","",IF(OR(O61&lt;&gt;"OK",P61&lt;&gt;"OK",Q61&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B61="","",IF(O61="Unresolved","Unresolved",IF(OR(O61&lt;&gt;"OK",P61&lt;&gt;"OK",Q61&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S61" s="14" t="str">
@@ -9114,7 +9172,7 @@
         <v/>
       </c>
       <c r="O62" s="14" t="str">
-        <f>IF(B62="","",IF(OR(C62="",L62=""),"Unmapped","OK"))</f>
+        <f>IF(B62="","",IF(L62="Unresolved","Unresolved",IF(OR(C62="",L62=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P62" s="14" t="str">
@@ -9126,7 +9184,7 @@
         <v/>
       </c>
       <c r="R62" s="14" t="str">
-        <f>IF(B62="","",IF(OR(O62&lt;&gt;"OK",P62&lt;&gt;"OK",Q62&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B62="","",IF(O62="Unresolved","Unresolved",IF(OR(O62&lt;&gt;"OK",P62&lt;&gt;"OK",Q62&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S62" s="14" t="str">
@@ -9192,7 +9250,7 @@
         <v/>
       </c>
       <c r="O63" s="14" t="str">
-        <f>IF(B63="","",IF(OR(C63="",L63=""),"Unmapped","OK"))</f>
+        <f>IF(B63="","",IF(L63="Unresolved","Unresolved",IF(OR(C63="",L63=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P63" s="14" t="str">
@@ -9204,7 +9262,7 @@
         <v/>
       </c>
       <c r="R63" s="14" t="str">
-        <f>IF(B63="","",IF(OR(O63&lt;&gt;"OK",P63&lt;&gt;"OK",Q63&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B63="","",IF(O63="Unresolved","Unresolved",IF(OR(O63&lt;&gt;"OK",P63&lt;&gt;"OK",Q63&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S63" s="14" t="str">
@@ -9270,7 +9328,7 @@
         <v/>
       </c>
       <c r="O64" s="14" t="str">
-        <f>IF(B64="","",IF(OR(C64="",L64=""),"Unmapped","OK"))</f>
+        <f>IF(B64="","",IF(L64="Unresolved","Unresolved",IF(OR(C64="",L64=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P64" s="14" t="str">
@@ -9282,7 +9340,7 @@
         <v/>
       </c>
       <c r="R64" s="14" t="str">
-        <f>IF(B64="","",IF(OR(O64&lt;&gt;"OK",P64&lt;&gt;"OK",Q64&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B64="","",IF(O64="Unresolved","Unresolved",IF(OR(O64&lt;&gt;"OK",P64&lt;&gt;"OK",Q64&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S64" s="14" t="str">
@@ -9348,7 +9406,7 @@
         <v/>
       </c>
       <c r="O65" s="14" t="str">
-        <f>IF(B65="","",IF(OR(C65="",L65=""),"Unmapped","OK"))</f>
+        <f>IF(B65="","",IF(L65="Unresolved","Unresolved",IF(OR(C65="",L65=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P65" s="14" t="str">
@@ -9360,7 +9418,7 @@
         <v/>
       </c>
       <c r="R65" s="14" t="str">
-        <f>IF(B65="","",IF(OR(O65&lt;&gt;"OK",P65&lt;&gt;"OK",Q65&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B65="","",IF(O65="Unresolved","Unresolved",IF(OR(O65&lt;&gt;"OK",P65&lt;&gt;"OK",Q65&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S65" s="14" t="str">
@@ -9426,7 +9484,7 @@
         <v/>
       </c>
       <c r="O66" s="14" t="str">
-        <f>IF(B66="","",IF(OR(C66="",L66=""),"Unmapped","OK"))</f>
+        <f>IF(B66="","",IF(L66="Unresolved","Unresolved",IF(OR(C66="",L66=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P66" s="14" t="str">
@@ -9438,7 +9496,7 @@
         <v/>
       </c>
       <c r="R66" s="14" t="str">
-        <f>IF(B66="","",IF(OR(O66&lt;&gt;"OK",P66&lt;&gt;"OK",Q66&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B66="","",IF(O66="Unresolved","Unresolved",IF(OR(O66&lt;&gt;"OK",P66&lt;&gt;"OK",Q66&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S66" s="14" t="str">
@@ -9504,7 +9562,7 @@
         <v/>
       </c>
       <c r="O67" s="14" t="str">
-        <f>IF(B67="","",IF(OR(C67="",L67=""),"Unmapped","OK"))</f>
+        <f>IF(B67="","",IF(L67="Unresolved","Unresolved",IF(OR(C67="",L67=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P67" s="14" t="str">
@@ -9516,7 +9574,7 @@
         <v/>
       </c>
       <c r="R67" s="14" t="str">
-        <f>IF(B67="","",IF(OR(O67&lt;&gt;"OK",P67&lt;&gt;"OK",Q67&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B67="","",IF(O67="Unresolved","Unresolved",IF(OR(O67&lt;&gt;"OK",P67&lt;&gt;"OK",Q67&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S67" s="14" t="str">
@@ -9582,7 +9640,7 @@
         <v/>
       </c>
       <c r="O68" s="14" t="str">
-        <f>IF(B68="","",IF(OR(C68="",L68=""),"Unmapped","OK"))</f>
+        <f>IF(B68="","",IF(L68="Unresolved","Unresolved",IF(OR(C68="",L68=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P68" s="14" t="str">
@@ -9594,7 +9652,7 @@
         <v/>
       </c>
       <c r="R68" s="14" t="str">
-        <f>IF(B68="","",IF(OR(O68&lt;&gt;"OK",P68&lt;&gt;"OK",Q68&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B68="","",IF(O68="Unresolved","Unresolved",IF(OR(O68&lt;&gt;"OK",P68&lt;&gt;"OK",Q68&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S68" s="14" t="str">
@@ -9660,7 +9718,7 @@
         <v/>
       </c>
       <c r="O69" s="14" t="str">
-        <f>IF(B69="","",IF(OR(C69="",L69=""),"Unmapped","OK"))</f>
+        <f>IF(B69="","",IF(L69="Unresolved","Unresolved",IF(OR(C69="",L69=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P69" s="14" t="str">
@@ -9672,7 +9730,7 @@
         <v/>
       </c>
       <c r="R69" s="14" t="str">
-        <f>IF(B69="","",IF(OR(O69&lt;&gt;"OK",P69&lt;&gt;"OK",Q69&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B69="","",IF(O69="Unresolved","Unresolved",IF(OR(O69&lt;&gt;"OK",P69&lt;&gt;"OK",Q69&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S69" s="14" t="str">
@@ -9738,7 +9796,7 @@
         <v/>
       </c>
       <c r="O70" s="14" t="str">
-        <f>IF(B70="","",IF(OR(C70="",L70=""),"Unmapped","OK"))</f>
+        <f>IF(B70="","",IF(L70="Unresolved","Unresolved",IF(OR(C70="",L70=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P70" s="14" t="str">
@@ -9750,7 +9808,7 @@
         <v/>
       </c>
       <c r="R70" s="14" t="str">
-        <f>IF(B70="","",IF(OR(O70&lt;&gt;"OK",P70&lt;&gt;"OK",Q70&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B70="","",IF(O70="Unresolved","Unresolved",IF(OR(O70&lt;&gt;"OK",P70&lt;&gt;"OK",Q70&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S70" s="14" t="str">
@@ -9816,7 +9874,7 @@
         <v/>
       </c>
       <c r="O71" s="14" t="str">
-        <f>IF(B71="","",IF(OR(C71="",L71=""),"Unmapped","OK"))</f>
+        <f>IF(B71="","",IF(L71="Unresolved","Unresolved",IF(OR(C71="",L71=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P71" s="14" t="str">
@@ -9828,7 +9886,7 @@
         <v/>
       </c>
       <c r="R71" s="14" t="str">
-        <f>IF(B71="","",IF(OR(O71&lt;&gt;"OK",P71&lt;&gt;"OK",Q71&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B71="","",IF(O71="Unresolved","Unresolved",IF(OR(O71&lt;&gt;"OK",P71&lt;&gt;"OK",Q71&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S71" s="14" t="str">
@@ -9894,7 +9952,7 @@
         <v/>
       </c>
       <c r="O72" s="14" t="str">
-        <f>IF(B72="","",IF(OR(C72="",L72=""),"Unmapped","OK"))</f>
+        <f>IF(B72="","",IF(L72="Unresolved","Unresolved",IF(OR(C72="",L72=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P72" s="14" t="str">
@@ -9906,7 +9964,7 @@
         <v/>
       </c>
       <c r="R72" s="14" t="str">
-        <f>IF(B72="","",IF(OR(O72&lt;&gt;"OK",P72&lt;&gt;"OK",Q72&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B72="","",IF(O72="Unresolved","Unresolved",IF(OR(O72&lt;&gt;"OK",P72&lt;&gt;"OK",Q72&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S72" s="14" t="str">
@@ -9972,7 +10030,7 @@
         <v/>
       </c>
       <c r="O73" s="14" t="str">
-        <f>IF(B73="","",IF(OR(C73="",L73=""),"Unmapped","OK"))</f>
+        <f>IF(B73="","",IF(L73="Unresolved","Unresolved",IF(OR(C73="",L73=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P73" s="14" t="str">
@@ -9984,7 +10042,7 @@
         <v/>
       </c>
       <c r="R73" s="14" t="str">
-        <f>IF(B73="","",IF(OR(O73&lt;&gt;"OK",P73&lt;&gt;"OK",Q73&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B73="","",IF(O73="Unresolved","Unresolved",IF(OR(O73&lt;&gt;"OK",P73&lt;&gt;"OK",Q73&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S73" s="14" t="str">
@@ -10050,7 +10108,7 @@
         <v/>
       </c>
       <c r="O74" s="14" t="str">
-        <f>IF(B74="","",IF(OR(C74="",L74=""),"Unmapped","OK"))</f>
+        <f>IF(B74="","",IF(L74="Unresolved","Unresolved",IF(OR(C74="",L74=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P74" s="14" t="str">
@@ -10062,7 +10120,7 @@
         <v/>
       </c>
       <c r="R74" s="14" t="str">
-        <f>IF(B74="","",IF(OR(O74&lt;&gt;"OK",P74&lt;&gt;"OK",Q74&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B74="","",IF(O74="Unresolved","Unresolved",IF(OR(O74&lt;&gt;"OK",P74&lt;&gt;"OK",Q74&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S74" s="14" t="str">
@@ -10128,7 +10186,7 @@
         <v/>
       </c>
       <c r="O75" s="14" t="str">
-        <f>IF(B75="","",IF(OR(C75="",L75=""),"Unmapped","OK"))</f>
+        <f>IF(B75="","",IF(L75="Unresolved","Unresolved",IF(OR(C75="",L75=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P75" s="14" t="str">
@@ -10140,7 +10198,7 @@
         <v/>
       </c>
       <c r="R75" s="14" t="str">
-        <f>IF(B75="","",IF(OR(O75&lt;&gt;"OK",P75&lt;&gt;"OK",Q75&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B75="","",IF(O75="Unresolved","Unresolved",IF(OR(O75&lt;&gt;"OK",P75&lt;&gt;"OK",Q75&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S75" s="14" t="str">
@@ -10206,7 +10264,7 @@
         <v/>
       </c>
       <c r="O76" s="14" t="str">
-        <f>IF(B76="","",IF(OR(C76="",L76=""),"Unmapped","OK"))</f>
+        <f>IF(B76="","",IF(L76="Unresolved","Unresolved",IF(OR(C76="",L76=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P76" s="14" t="str">
@@ -10218,7 +10276,7 @@
         <v/>
       </c>
       <c r="R76" s="14" t="str">
-        <f>IF(B76="","",IF(OR(O76&lt;&gt;"OK",P76&lt;&gt;"OK",Q76&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B76="","",IF(O76="Unresolved","Unresolved",IF(OR(O76&lt;&gt;"OK",P76&lt;&gt;"OK",Q76&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S76" s="14" t="str">
@@ -10284,7 +10342,7 @@
         <v/>
       </c>
       <c r="O77" s="14" t="str">
-        <f>IF(B77="","",IF(OR(C77="",L77=""),"Unmapped","OK"))</f>
+        <f>IF(B77="","",IF(L77="Unresolved","Unresolved",IF(OR(C77="",L77=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P77" s="14" t="str">
@@ -10296,7 +10354,7 @@
         <v/>
       </c>
       <c r="R77" s="14" t="str">
-        <f>IF(B77="","",IF(OR(O77&lt;&gt;"OK",P77&lt;&gt;"OK",Q77&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B77="","",IF(O77="Unresolved","Unresolved",IF(OR(O77&lt;&gt;"OK",P77&lt;&gt;"OK",Q77&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S77" s="14" t="str">
@@ -10362,7 +10420,7 @@
         <v/>
       </c>
       <c r="O78" s="14" t="str">
-        <f>IF(B78="","",IF(OR(C78="",L78=""),"Unmapped","OK"))</f>
+        <f>IF(B78="","",IF(L78="Unresolved","Unresolved",IF(OR(C78="",L78=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P78" s="14" t="str">
@@ -10374,7 +10432,7 @@
         <v/>
       </c>
       <c r="R78" s="14" t="str">
-        <f>IF(B78="","",IF(OR(O78&lt;&gt;"OK",P78&lt;&gt;"OK",Q78&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B78="","",IF(O78="Unresolved","Unresolved",IF(OR(O78&lt;&gt;"OK",P78&lt;&gt;"OK",Q78&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S78" s="14" t="str">
@@ -10440,7 +10498,7 @@
         <v/>
       </c>
       <c r="O79" s="14" t="str">
-        <f>IF(B79="","",IF(OR(C79="",L79=""),"Unmapped","OK"))</f>
+        <f>IF(B79="","",IF(L79="Unresolved","Unresolved",IF(OR(C79="",L79=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P79" s="14" t="str">
@@ -10452,7 +10510,7 @@
         <v/>
       </c>
       <c r="R79" s="14" t="str">
-        <f>IF(B79="","",IF(OR(O79&lt;&gt;"OK",P79&lt;&gt;"OK",Q79&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B79="","",IF(O79="Unresolved","Unresolved",IF(OR(O79&lt;&gt;"OK",P79&lt;&gt;"OK",Q79&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S79" s="14" t="str">
@@ -10518,7 +10576,7 @@
         <v/>
       </c>
       <c r="O80" s="14" t="str">
-        <f>IF(B80="","",IF(OR(C80="",L80=""),"Unmapped","OK"))</f>
+        <f>IF(B80="","",IF(L80="Unresolved","Unresolved",IF(OR(C80="",L80=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P80" s="14" t="str">
@@ -10530,7 +10588,7 @@
         <v/>
       </c>
       <c r="R80" s="14" t="str">
-        <f>IF(B80="","",IF(OR(O80&lt;&gt;"OK",P80&lt;&gt;"OK",Q80&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B80="","",IF(O80="Unresolved","Unresolved",IF(OR(O80&lt;&gt;"OK",P80&lt;&gt;"OK",Q80&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S80" s="14" t="str">
@@ -10596,7 +10654,7 @@
         <v/>
       </c>
       <c r="O81" s="14" t="str">
-        <f>IF(B81="","",IF(OR(C81="",L81=""),"Unmapped","OK"))</f>
+        <f>IF(B81="","",IF(L81="Unresolved","Unresolved",IF(OR(C81="",L81=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P81" s="14" t="str">
@@ -10608,7 +10666,7 @@
         <v/>
       </c>
       <c r="R81" s="14" t="str">
-        <f>IF(B81="","",IF(OR(O81&lt;&gt;"OK",P81&lt;&gt;"OK",Q81&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B81="","",IF(O81="Unresolved","Unresolved",IF(OR(O81&lt;&gt;"OK",P81&lt;&gt;"OK",Q81&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S81" s="14" t="str">
@@ -10674,7 +10732,7 @@
         <v/>
       </c>
       <c r="O82" s="14" t="str">
-        <f>IF(B82="","",IF(OR(C82="",L82=""),"Unmapped","OK"))</f>
+        <f>IF(B82="","",IF(L82="Unresolved","Unresolved",IF(OR(C82="",L82=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P82" s="14" t="str">
@@ -10686,7 +10744,7 @@
         <v/>
       </c>
       <c r="R82" s="14" t="str">
-        <f>IF(B82="","",IF(OR(O82&lt;&gt;"OK",P82&lt;&gt;"OK",Q82&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B82="","",IF(O82="Unresolved","Unresolved",IF(OR(O82&lt;&gt;"OK",P82&lt;&gt;"OK",Q82&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S82" s="14" t="str">
@@ -10752,7 +10810,7 @@
         <v/>
       </c>
       <c r="O83" s="14" t="str">
-        <f>IF(B83="","",IF(OR(C83="",L83=""),"Unmapped","OK"))</f>
+        <f>IF(B83="","",IF(L83="Unresolved","Unresolved",IF(OR(C83="",L83=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P83" s="14" t="str">
@@ -10764,7 +10822,7 @@
         <v/>
       </c>
       <c r="R83" s="14" t="str">
-        <f>IF(B83="","",IF(OR(O83&lt;&gt;"OK",P83&lt;&gt;"OK",Q83&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B83="","",IF(O83="Unresolved","Unresolved",IF(OR(O83&lt;&gt;"OK",P83&lt;&gt;"OK",Q83&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S83" s="14" t="str">
@@ -10830,7 +10888,7 @@
         <v/>
       </c>
       <c r="O84" s="14" t="str">
-        <f>IF(B84="","",IF(OR(C84="",L84=""),"Unmapped","OK"))</f>
+        <f>IF(B84="","",IF(L84="Unresolved","Unresolved",IF(OR(C84="",L84=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P84" s="14" t="str">
@@ -10842,7 +10900,7 @@
         <v/>
       </c>
       <c r="R84" s="14" t="str">
-        <f>IF(B84="","",IF(OR(O84&lt;&gt;"OK",P84&lt;&gt;"OK",Q84&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B84="","",IF(O84="Unresolved","Unresolved",IF(OR(O84&lt;&gt;"OK",P84&lt;&gt;"OK",Q84&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S84" s="14" t="str">
@@ -10908,7 +10966,7 @@
         <v/>
       </c>
       <c r="O85" s="14" t="str">
-        <f>IF(B85="","",IF(OR(C85="",L85=""),"Unmapped","OK"))</f>
+        <f>IF(B85="","",IF(L85="Unresolved","Unresolved",IF(OR(C85="",L85=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P85" s="14" t="str">
@@ -10920,7 +10978,7 @@
         <v/>
       </c>
       <c r="R85" s="14" t="str">
-        <f>IF(B85="","",IF(OR(O85&lt;&gt;"OK",P85&lt;&gt;"OK",Q85&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B85="","",IF(O85="Unresolved","Unresolved",IF(OR(O85&lt;&gt;"OK",P85&lt;&gt;"OK",Q85&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S85" s="14" t="str">
@@ -10986,7 +11044,7 @@
         <v/>
       </c>
       <c r="O86" s="14" t="str">
-        <f>IF(B86="","",IF(OR(C86="",L86=""),"Unmapped","OK"))</f>
+        <f>IF(B86="","",IF(L86="Unresolved","Unresolved",IF(OR(C86="",L86=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P86" s="14" t="str">
@@ -10998,7 +11056,7 @@
         <v/>
       </c>
       <c r="R86" s="14" t="str">
-        <f>IF(B86="","",IF(OR(O86&lt;&gt;"OK",P86&lt;&gt;"OK",Q86&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B86="","",IF(O86="Unresolved","Unresolved",IF(OR(O86&lt;&gt;"OK",P86&lt;&gt;"OK",Q86&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S86" s="14" t="str">
@@ -11064,7 +11122,7 @@
         <v/>
       </c>
       <c r="O87" s="14" t="str">
-        <f>IF(B87="","",IF(OR(C87="",L87=""),"Unmapped","OK"))</f>
+        <f>IF(B87="","",IF(L87="Unresolved","Unresolved",IF(OR(C87="",L87=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P87" s="14" t="str">
@@ -11076,7 +11134,7 @@
         <v/>
       </c>
       <c r="R87" s="14" t="str">
-        <f>IF(B87="","",IF(OR(O87&lt;&gt;"OK",P87&lt;&gt;"OK",Q87&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B87="","",IF(O87="Unresolved","Unresolved",IF(OR(O87&lt;&gt;"OK",P87&lt;&gt;"OK",Q87&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S87" s="14" t="str">
@@ -11142,7 +11200,7 @@
         <v/>
       </c>
       <c r="O88" s="14" t="str">
-        <f>IF(B88="","",IF(OR(C88="",L88=""),"Unmapped","OK"))</f>
+        <f>IF(B88="","",IF(L88="Unresolved","Unresolved",IF(OR(C88="",L88=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P88" s="14" t="str">
@@ -11154,7 +11212,7 @@
         <v/>
       </c>
       <c r="R88" s="14" t="str">
-        <f>IF(B88="","",IF(OR(O88&lt;&gt;"OK",P88&lt;&gt;"OK",Q88&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B88="","",IF(O88="Unresolved","Unresolved",IF(OR(O88&lt;&gt;"OK",P88&lt;&gt;"OK",Q88&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S88" s="14" t="str">
@@ -11220,7 +11278,7 @@
         <v/>
       </c>
       <c r="O89" s="14" t="str">
-        <f>IF(B89="","",IF(OR(C89="",L89=""),"Unmapped","OK"))</f>
+        <f>IF(B89="","",IF(L89="Unresolved","Unresolved",IF(OR(C89="",L89=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P89" s="14" t="str">
@@ -11232,7 +11290,7 @@
         <v/>
       </c>
       <c r="R89" s="14" t="str">
-        <f>IF(B89="","",IF(OR(O89&lt;&gt;"OK",P89&lt;&gt;"OK",Q89&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B89="","",IF(O89="Unresolved","Unresolved",IF(OR(O89&lt;&gt;"OK",P89&lt;&gt;"OK",Q89&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S89" s="14" t="str">
@@ -11298,7 +11356,7 @@
         <v/>
       </c>
       <c r="O90" s="14" t="str">
-        <f>IF(B90="","",IF(OR(C90="",L90=""),"Unmapped","OK"))</f>
+        <f>IF(B90="","",IF(L90="Unresolved","Unresolved",IF(OR(C90="",L90=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P90" s="14" t="str">
@@ -11310,7 +11368,7 @@
         <v/>
       </c>
       <c r="R90" s="14" t="str">
-        <f>IF(B90="","",IF(OR(O90&lt;&gt;"OK",P90&lt;&gt;"OK",Q90&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B90="","",IF(O90="Unresolved","Unresolved",IF(OR(O90&lt;&gt;"OK",P90&lt;&gt;"OK",Q90&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S90" s="14" t="str">
@@ -11376,7 +11434,7 @@
         <v/>
       </c>
       <c r="O91" s="14" t="str">
-        <f>IF(B91="","",IF(OR(C91="",L91=""),"Unmapped","OK"))</f>
+        <f>IF(B91="","",IF(L91="Unresolved","Unresolved",IF(OR(C91="",L91=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P91" s="14" t="str">
@@ -11388,7 +11446,7 @@
         <v/>
       </c>
       <c r="R91" s="14" t="str">
-        <f>IF(B91="","",IF(OR(O91&lt;&gt;"OK",P91&lt;&gt;"OK",Q91&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B91="","",IF(O91="Unresolved","Unresolved",IF(OR(O91&lt;&gt;"OK",P91&lt;&gt;"OK",Q91&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S91" s="14" t="str">
@@ -11454,7 +11512,7 @@
         <v/>
       </c>
       <c r="O92" s="14" t="str">
-        <f>IF(B92="","",IF(OR(C92="",L92=""),"Unmapped","OK"))</f>
+        <f>IF(B92="","",IF(L92="Unresolved","Unresolved",IF(OR(C92="",L92=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P92" s="14" t="str">
@@ -11466,7 +11524,7 @@
         <v/>
       </c>
       <c r="R92" s="14" t="str">
-        <f>IF(B92="","",IF(OR(O92&lt;&gt;"OK",P92&lt;&gt;"OK",Q92&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B92="","",IF(O92="Unresolved","Unresolved",IF(OR(O92&lt;&gt;"OK",P92&lt;&gt;"OK",Q92&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S92" s="14" t="str">
@@ -11532,7 +11590,7 @@
         <v/>
       </c>
       <c r="O93" s="14" t="str">
-        <f>IF(B93="","",IF(OR(C93="",L93=""),"Unmapped","OK"))</f>
+        <f>IF(B93="","",IF(L93="Unresolved","Unresolved",IF(OR(C93="",L93=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P93" s="14" t="str">
@@ -11544,7 +11602,7 @@
         <v/>
       </c>
       <c r="R93" s="14" t="str">
-        <f>IF(B93="","",IF(OR(O93&lt;&gt;"OK",P93&lt;&gt;"OK",Q93&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B93="","",IF(O93="Unresolved","Unresolved",IF(OR(O93&lt;&gt;"OK",P93&lt;&gt;"OK",Q93&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S93" s="14" t="str">
@@ -11610,7 +11668,7 @@
         <v/>
       </c>
       <c r="O94" s="14" t="str">
-        <f>IF(B94="","",IF(OR(C94="",L94=""),"Unmapped","OK"))</f>
+        <f>IF(B94="","",IF(L94="Unresolved","Unresolved",IF(OR(C94="",L94=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P94" s="14" t="str">
@@ -11622,7 +11680,7 @@
         <v/>
       </c>
       <c r="R94" s="14" t="str">
-        <f>IF(B94="","",IF(OR(O94&lt;&gt;"OK",P94&lt;&gt;"OK",Q94&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B94="","",IF(O94="Unresolved","Unresolved",IF(OR(O94&lt;&gt;"OK",P94&lt;&gt;"OK",Q94&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S94" s="14" t="str">
@@ -11688,7 +11746,7 @@
         <v/>
       </c>
       <c r="O95" s="14" t="str">
-        <f>IF(B95="","",IF(OR(C95="",L95=""),"Unmapped","OK"))</f>
+        <f>IF(B95="","",IF(L95="Unresolved","Unresolved",IF(OR(C95="",L95=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P95" s="14" t="str">
@@ -11700,7 +11758,7 @@
         <v/>
       </c>
       <c r="R95" s="14" t="str">
-        <f>IF(B95="","",IF(OR(O95&lt;&gt;"OK",P95&lt;&gt;"OK",Q95&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B95="","",IF(O95="Unresolved","Unresolved",IF(OR(O95&lt;&gt;"OK",P95&lt;&gt;"OK",Q95&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S95" s="14" t="str">
@@ -11766,7 +11824,7 @@
         <v/>
       </c>
       <c r="O96" s="14" t="str">
-        <f>IF(B96="","",IF(OR(C96="",L96=""),"Unmapped","OK"))</f>
+        <f>IF(B96="","",IF(L96="Unresolved","Unresolved",IF(OR(C96="",L96=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P96" s="14" t="str">
@@ -11778,7 +11836,7 @@
         <v/>
       </c>
       <c r="R96" s="14" t="str">
-        <f>IF(B96="","",IF(OR(O96&lt;&gt;"OK",P96&lt;&gt;"OK",Q96&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B96="","",IF(O96="Unresolved","Unresolved",IF(OR(O96&lt;&gt;"OK",P96&lt;&gt;"OK",Q96&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S96" s="14" t="str">
@@ -11844,7 +11902,7 @@
         <v/>
       </c>
       <c r="O97" s="14" t="str">
-        <f>IF(B97="","",IF(OR(C97="",L97=""),"Unmapped","OK"))</f>
+        <f>IF(B97="","",IF(L97="Unresolved","Unresolved",IF(OR(C97="",L97=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P97" s="14" t="str">
@@ -11856,7 +11914,7 @@
         <v/>
       </c>
       <c r="R97" s="14" t="str">
-        <f>IF(B97="","",IF(OR(O97&lt;&gt;"OK",P97&lt;&gt;"OK",Q97&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B97="","",IF(O97="Unresolved","Unresolved",IF(OR(O97&lt;&gt;"OK",P97&lt;&gt;"OK",Q97&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S97" s="14" t="str">
@@ -11922,7 +11980,7 @@
         <v/>
       </c>
       <c r="O98" s="14" t="str">
-        <f>IF(B98="","",IF(OR(C98="",L98=""),"Unmapped","OK"))</f>
+        <f>IF(B98="","",IF(L98="Unresolved","Unresolved",IF(OR(C98="",L98=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P98" s="14" t="str">
@@ -11934,7 +11992,7 @@
         <v/>
       </c>
       <c r="R98" s="14" t="str">
-        <f>IF(B98="","",IF(OR(O98&lt;&gt;"OK",P98&lt;&gt;"OK",Q98&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B98="","",IF(O98="Unresolved","Unresolved",IF(OR(O98&lt;&gt;"OK",P98&lt;&gt;"OK",Q98&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S98" s="14" t="str">
@@ -12000,7 +12058,7 @@
         <v/>
       </c>
       <c r="O99" s="14" t="str">
-        <f>IF(B99="","",IF(OR(C99="",L99=""),"Unmapped","OK"))</f>
+        <f>IF(B99="","",IF(L99="Unresolved","Unresolved",IF(OR(C99="",L99=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P99" s="14" t="str">
@@ -12012,7 +12070,7 @@
         <v/>
       </c>
       <c r="R99" s="14" t="str">
-        <f>IF(B99="","",IF(OR(O99&lt;&gt;"OK",P99&lt;&gt;"OK",Q99&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B99="","",IF(O99="Unresolved","Unresolved",IF(OR(O99&lt;&gt;"OK",P99&lt;&gt;"OK",Q99&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S99" s="14" t="str">
@@ -12078,7 +12136,7 @@
         <v/>
       </c>
       <c r="O100" s="14" t="str">
-        <f>IF(B100="","",IF(OR(C100="",L100=""),"Unmapped","OK"))</f>
+        <f>IF(B100="","",IF(L100="Unresolved","Unresolved",IF(OR(C100="",L100=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P100" s="14" t="str">
@@ -12090,7 +12148,7 @@
         <v/>
       </c>
       <c r="R100" s="14" t="str">
-        <f>IF(B100="","",IF(OR(O100&lt;&gt;"OK",P100&lt;&gt;"OK",Q100&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B100="","",IF(O100="Unresolved","Unresolved",IF(OR(O100&lt;&gt;"OK",P100&lt;&gt;"OK",Q100&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S100" s="14" t="str">
@@ -12156,7 +12214,7 @@
         <v/>
       </c>
       <c r="O101" s="14" t="str">
-        <f>IF(B101="","",IF(OR(C101="",L101=""),"Unmapped","OK"))</f>
+        <f>IF(B101="","",IF(L101="Unresolved","Unresolved",IF(OR(C101="",L101=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P101" s="14" t="str">
@@ -12168,7 +12226,7 @@
         <v/>
       </c>
       <c r="R101" s="14" t="str">
-        <f>IF(B101="","",IF(OR(O101&lt;&gt;"OK",P101&lt;&gt;"OK",Q101&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B101="","",IF(O101="Unresolved","Unresolved",IF(OR(O101&lt;&gt;"OK",P101&lt;&gt;"OK",Q101&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S101" s="14" t="str">
@@ -12234,7 +12292,7 @@
         <v/>
       </c>
       <c r="O102" s="14" t="str">
-        <f>IF(B102="","",IF(OR(C102="",L102=""),"Unmapped","OK"))</f>
+        <f>IF(B102="","",IF(L102="Unresolved","Unresolved",IF(OR(C102="",L102=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P102" s="14" t="str">
@@ -12246,7 +12304,7 @@
         <v/>
       </c>
       <c r="R102" s="14" t="str">
-        <f>IF(B102="","",IF(OR(O102&lt;&gt;"OK",P102&lt;&gt;"OK",Q102&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B102="","",IF(O102="Unresolved","Unresolved",IF(OR(O102&lt;&gt;"OK",P102&lt;&gt;"OK",Q102&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S102" s="14" t="str">
@@ -12312,7 +12370,7 @@
         <v/>
       </c>
       <c r="O103" s="14" t="str">
-        <f>IF(B103="","",IF(OR(C103="",L103=""),"Unmapped","OK"))</f>
+        <f>IF(B103="","",IF(L103="Unresolved","Unresolved",IF(OR(C103="",L103=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P103" s="14" t="str">
@@ -12324,7 +12382,7 @@
         <v/>
       </c>
       <c r="R103" s="14" t="str">
-        <f>IF(B103="","",IF(OR(O103&lt;&gt;"OK",P103&lt;&gt;"OK",Q103&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B103="","",IF(O103="Unresolved","Unresolved",IF(OR(O103&lt;&gt;"OK",P103&lt;&gt;"OK",Q103&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S103" s="14" t="str">
@@ -12390,7 +12448,7 @@
         <v/>
       </c>
       <c r="O104" s="14" t="str">
-        <f>IF(B104="","",IF(OR(C104="",L104=""),"Unmapped","OK"))</f>
+        <f>IF(B104="","",IF(L104="Unresolved","Unresolved",IF(OR(C104="",L104=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P104" s="14" t="str">
@@ -12402,7 +12460,7 @@
         <v/>
       </c>
       <c r="R104" s="14" t="str">
-        <f>IF(B104="","",IF(OR(O104&lt;&gt;"OK",P104&lt;&gt;"OK",Q104&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B104="","",IF(O104="Unresolved","Unresolved",IF(OR(O104&lt;&gt;"OK",P104&lt;&gt;"OK",Q104&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S104" s="14" t="str">
@@ -12468,7 +12526,7 @@
         <v/>
       </c>
       <c r="O105" s="14" t="str">
-        <f>IF(B105="","",IF(OR(C105="",L105=""),"Unmapped","OK"))</f>
+        <f>IF(B105="","",IF(L105="Unresolved","Unresolved",IF(OR(C105="",L105=""),"Unmapped","OK")))</f>
         <v/>
       </c>
       <c r="P105" s="14" t="str">
@@ -12480,7 +12538,7 @@
         <v/>
       </c>
       <c r="R105" s="14" t="str">
-        <f>IF(B105="","",IF(OR(O105&lt;&gt;"OK",P105&lt;&gt;"OK",Q105&lt;&gt;"OK"),"Review","Complete"))</f>
+        <f>IF(B105="","",IF(O105="Unresolved","Unresolved",IF(OR(O105&lt;&gt;"OK",P105&lt;&gt;"OK",Q105&lt;&gt;"OK"),"Review","Complete")))</f>
         <v/>
       </c>
       <c r="S105" s="14" t="str">
@@ -12505,60 +12563,72 @@
       <formula>NOT(ISERROR(SEARCH("Unusual",O6)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="3" priority="4">
+      <formula>NOT(ISERROR(SEARCH("Unresolved",O6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="5">
       <formula>NOT(ISERROR(SEARCH("OK",O6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="5">
+    <cfRule type="containsText" dxfId="5" priority="6">
       <formula>NOT(ISERROR(SEARCH("Complete",O6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P6:P105">
-    <cfRule type="containsText" dxfId="5" priority="6">
+    <cfRule type="containsText" dxfId="6" priority="7">
       <formula>NOT(ISERROR(SEARCH("Review",P6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="7">
+    <cfRule type="containsText" dxfId="7" priority="8">
       <formula>NOT(ISERROR(SEARCH("Unmapped",P6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="8">
+    <cfRule type="containsText" dxfId="8" priority="9">
       <formula>NOT(ISERROR(SEARCH("Unusual",P6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="9">
+    <cfRule type="containsText" dxfId="9" priority="10">
+      <formula>NOT(ISERROR(SEARCH("Unresolved",P6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="10" priority="11">
       <formula>NOT(ISERROR(SEARCH("OK",P6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="10">
+    <cfRule type="containsText" dxfId="11" priority="12">
       <formula>NOT(ISERROR(SEARCH("Complete",P6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q6:Q105">
-    <cfRule type="containsText" dxfId="10" priority="11">
+    <cfRule type="containsText" dxfId="12" priority="13">
       <formula>NOT(ISERROR(SEARCH("Review",Q6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="12">
+    <cfRule type="containsText" dxfId="13" priority="14">
       <formula>NOT(ISERROR(SEARCH("Unmapped",Q6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="13">
+    <cfRule type="containsText" dxfId="14" priority="15">
       <formula>NOT(ISERROR(SEARCH("Unusual",Q6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="14">
+    <cfRule type="containsText" dxfId="15" priority="16">
+      <formula>NOT(ISERROR(SEARCH("Unresolved",Q6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="16" priority="17">
       <formula>NOT(ISERROR(SEARCH("OK",Q6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="15">
+    <cfRule type="containsText" dxfId="17" priority="18">
       <formula>NOT(ISERROR(SEARCH("Complete",Q6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R6:R105">
-    <cfRule type="containsText" dxfId="15" priority="16">
+    <cfRule type="containsText" dxfId="18" priority="19">
       <formula>NOT(ISERROR(SEARCH("Review",R6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="17">
+    <cfRule type="containsText" dxfId="19" priority="20">
       <formula>NOT(ISERROR(SEARCH("Unmapped",R6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="18">
+    <cfRule type="containsText" dxfId="20" priority="21">
       <formula>NOT(ISERROR(SEARCH("Unusual",R6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="19">
+    <cfRule type="containsText" dxfId="21" priority="22">
+      <formula>NOT(ISERROR(SEARCH("Unresolved",R6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="22" priority="23">
       <formula>NOT(ISERROR(SEARCH("OK",R6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="19" priority="20">
+    <cfRule type="containsText" dxfId="23" priority="24">
       <formula>NOT(ISERROR(SEARCH("Complete",R6)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12586,7 +12656,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -12608,7 +12678,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -12621,7 +12691,7 @@
     <row r="4" spans="1:8" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B5" s="17" t="str">
         <f>'Start Here'!B4</f>
@@ -12642,10 +12712,10 @@
         <v>Taylor Morgan</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H5" s="19" t="str">
-        <f>IF(AND(ABS(D12)&lt;0.01,F15=0),"Complete","Review")</f>
+        <f>IF(AND(ABS(D15)&lt;0.01,H18=0),"Complete","Review")</f>
         <v>Review</v>
       </c>
     </row>
@@ -12653,15 +12723,15 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.25"/>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D8" s="17"/>
       <c r="E8" s="20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -12684,103 +12754,122 @@
     <row r="10" spans="1:8" x14ac:dyDescent="0.25"/>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D11" s="17"/>
       <c r="E11" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="17"/>
       <c r="B12" s="21">
-        <f>SUM('Review'!$M$6:$M$105)</f>
-        <v>0</v>
+        <f>SUM('Review'!$F$6:$F$105)</f>
+        <v>395000</v>
       </c>
       <c r="C12" s="17"/>
       <c r="D12" s="21">
-        <f>F9+B12</f>
-        <v>0</v>
+        <f>SUM('Review'!$G$6:$G$105)</f>
+        <v>395000</v>
       </c>
       <c r="E12" s="17"/>
-      <c r="F12" s="22">
-        <f>COUNTIF('Review'!$Q$6:$Q$105,"Review")</f>
-        <v>9</v>
+      <c r="F12" s="21">
+        <f>B12-D12</f>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B14" s="17"/>
       <c r="C14" s="20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D14" s="17"/>
       <c r="E14" s="20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="17"/>
-      <c r="B15" s="22">
+      <c r="B15" s="21">
+        <f>SUM('Review'!$M$6:$M$105)</f>
+        <v>0</v>
+      </c>
+      <c r="C15" s="17"/>
+      <c r="D15" s="21">
+        <f>F9+B15</f>
+        <v>0</v>
+      </c>
+      <c r="E15" s="17"/>
+      <c r="F15" s="22">
+        <f>COUNTIF('Review'!$Q$6:$Q$105,"Review")</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="17"/>
+      <c r="C17" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="D17" s="17"/>
+      <c r="E17" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="F17" s="17"/>
+      <c r="G17" s="20" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="17"/>
+      <c r="B18" s="22">
         <f>COUNTIF('Review'!$P$6:$P$105,"Unusual")</f>
         <v>1</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="22">
+      <c r="C18" s="17"/>
+      <c r="D18" s="22">
         <f>COUNTIF('Review'!$O$6:$O$105,"Unmapped")</f>
         <v>1</v>
       </c>
-      <c r="E15" s="17"/>
-      <c r="F15" s="22">
-        <f>COUNTIF('Review'!$R$6:$R$105,"Review")</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="23"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
-        <v>112</v>
-      </c>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-    </row>
+      <c r="E18" s="17"/>
+      <c r="F18" s="22">
+        <f>COUNTIF('Review'!$R$6:$R$105,"Unresolved")</f>
+        <v>1</v>
+      </c>
+      <c r="G18" s="17"/>
+      <c r="H18" s="22">
+        <f>COUNTIF('Review'!$R$6:$R$105,"Review")+COUNTIF('Review'!$R$6:$R$105,"Unresolved")</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="24"/>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
+      <c r="A20" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="24"/>
+      <c r="A21" s="24" t="s">
+        <v>117</v>
+      </c>
       <c r="B21" s="24"/>
       <c r="C21" s="24"/>
       <c r="D21" s="24"/>
@@ -12799,20 +12888,29 @@
       <c r="G22" s="24"/>
       <c r="H22" s="24"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="24"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+    </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:H2"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A19:H22"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A21:H23"/>
   </mergeCells>
   <conditionalFormatting sqref="H5">
-    <cfRule type="expression" dxfId="20" priority="1">
+    <cfRule type="expression" dxfId="24" priority="1">
       <formula>H5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="2">
+    <cfRule type="expression" dxfId="25" priority="2">
       <formula>H5="Complete"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12823,7 +12921,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -12840,7 +12938,7 @@
         <v>35</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>7</v>
@@ -12854,7 +12952,7 @@
         <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -12862,76 +12960,84 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
         <v>45</v>
       </c>
       <c r="C3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B4" t="s">
         <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B5" t="s">
         <v>56</v>
       </c>
       <c r="C5" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C6" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" t="s">
         <v>52</v>
-      </c>
-      <c r="B7" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
         <v>52</v>
       </c>
     </row>

</xml_diff>